<commit_message>
Fix #NAME? errors: replace dot-notation functions with compatible equivalents in 06_Forecasting.xlsx
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-12/06_Forecasting.xlsx
+++ b/rFLA300/chapter-12/06_Forecasting.xlsx
@@ -108,7 +108,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -122,11 +122,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -192,6 +220,8 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -583,6 +613,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1505,6 +1536,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1555,11 +1587,11 @@
         <v>55.9</v>
       </c>
       <c r="D5" s="10">
-        <f>FORECAST.LINEAR(A5,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A5,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>FORECAST.ETS(A5,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A5,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F5" s="10">
@@ -1585,11 +1617,11 @@
         <v>52.7</v>
       </c>
       <c r="D6" s="10">
-        <f>FORECAST.LINEAR(A6,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A6,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E6" s="10">
-        <f>FORECAST.ETS(A6,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A6,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F6" s="10">
@@ -1615,11 +1647,11 @@
         <v>60.8</v>
       </c>
       <c r="D7" s="10">
-        <f>FORECAST.LINEAR(A7,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A7,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>FORECAST.ETS(A7,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A7,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F7" s="10">
@@ -1645,11 +1677,11 @@
         <v>63.6</v>
       </c>
       <c r="D8" s="10">
-        <f>FORECAST.LINEAR(A8,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A8,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E8" s="10">
-        <f>FORECAST.ETS(A8,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A8,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F8" s="10">
@@ -1675,11 +1707,11 @@
         <v>68.09999999999999</v>
       </c>
       <c r="D9" s="10">
-        <f>FORECAST.LINEAR(A9,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A9,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>FORECAST.ETS(A9,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A9,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F9" s="10">
@@ -1705,11 +1737,11 @@
         <v>70.8</v>
       </c>
       <c r="D10" s="10">
-        <f>FORECAST.LINEAR(A10,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A10,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E10" s="10">
-        <f>FORECAST.ETS(A10,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A10,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F10" s="10">
@@ -1735,11 +1767,11 @@
         <v>76.40000000000001</v>
       </c>
       <c r="D11" s="10">
-        <f>FORECAST.LINEAR(A11,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A11,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>FORECAST.ETS(A11,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A11,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F11" s="10">
@@ -1765,11 +1797,11 @@
         <v>77.40000000000001</v>
       </c>
       <c r="D12" s="10">
-        <f>FORECAST.LINEAR(A12,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A12,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E12" s="10">
-        <f>FORECAST.ETS(A12,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A12,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F12" s="10">
@@ -1795,11 +1827,11 @@
         <v>70.40000000000001</v>
       </c>
       <c r="D13" s="10">
-        <f>FORECAST.LINEAR(A13,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A13,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>FORECAST.ETS(A13,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A13,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F13" s="10">
@@ -1825,11 +1857,11 @@
         <v>69.8</v>
       </c>
       <c r="D14" s="10">
-        <f>FORECAST.LINEAR(A14,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A14,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E14" s="10">
-        <f>FORECAST.ETS(A14,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A14,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F14" s="10">
@@ -1855,11 +1887,11 @@
         <v>80.8</v>
       </c>
       <c r="D15" s="10">
-        <f>FORECAST.LINEAR(A15,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A15,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>FORECAST.ETS(A15,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A15,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F15" s="10">
@@ -1885,11 +1917,11 @@
         <v>100.9</v>
       </c>
       <c r="D16" s="10">
-        <f>FORECAST.LINEAR(A16,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A16,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E16" s="10">
-        <f>FORECAST.ETS(A16,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A16,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F16" s="10">
@@ -1915,11 +1947,11 @@
         <v>65.59999999999999</v>
       </c>
       <c r="D17" s="10">
-        <f>FORECAST.LINEAR(A17,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A17,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>FORECAST.ETS(A17,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A17,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F17" s="10">
@@ -1945,11 +1977,11 @@
         <v>60.6</v>
       </c>
       <c r="D18" s="10">
-        <f>FORECAST.LINEAR(A18,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A18,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>FORECAST.ETS(A18,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A18,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F18" s="10">
@@ -1975,11 +2007,11 @@
         <v>68.7</v>
       </c>
       <c r="D19" s="10">
-        <f>FORECAST.LINEAR(A19,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A19,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>FORECAST.ETS(A19,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A19,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F19" s="10">
@@ -2005,11 +2037,11 @@
         <v>71.5</v>
       </c>
       <c r="D20" s="10">
-        <f>FORECAST.LINEAR(A20,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A20,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E20" s="10">
-        <f>FORECAST.ETS(A20,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A20,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F20" s="10">
@@ -2035,11 +2067,11 @@
         <v>80.90000000000001</v>
       </c>
       <c r="D21" s="10">
-        <f>FORECAST.LINEAR(A21,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A21,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>FORECAST.ETS(A21,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A21,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F21" s="10">
@@ -2065,11 +2097,11 @@
         <v>82.90000000000001</v>
       </c>
       <c r="D22" s="10">
-        <f>FORECAST.LINEAR(A22,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A22,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>FORECAST.ETS(A22,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A22,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F22" s="10">
@@ -2095,11 +2127,11 @@
         <v>86.2</v>
       </c>
       <c r="D23" s="10">
-        <f>FORECAST.LINEAR(A23,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A23,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>FORECAST.ETS(A23,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A23,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F23" s="10">
@@ -2125,11 +2157,11 @@
         <v>86.90000000000001</v>
       </c>
       <c r="D24" s="10">
-        <f>FORECAST.LINEAR(A24,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A24,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E24" s="10">
-        <f>FORECAST.ETS(A24,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A24,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F24" s="10">
@@ -2155,11 +2187,11 @@
         <v>80.8</v>
       </c>
       <c r="D25" s="10">
-        <f>FORECAST.LINEAR(A25,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A25,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E25" s="10">
-        <f>FORECAST.ETS(A25,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A25,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F25" s="10">
@@ -2185,11 +2217,11 @@
         <v>79.09999999999999</v>
       </c>
       <c r="D26" s="10">
-        <f>FORECAST.LINEAR(A26,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A26,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E26" s="10">
-        <f>FORECAST.ETS(A26,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A26,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F26" s="10">
@@ -2215,11 +2247,11 @@
         <v>90.59999999999999</v>
       </c>
       <c r="D27" s="10">
-        <f>FORECAST.LINEAR(A27,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A27,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E27" s="10">
-        <f>FORECAST.ETS(A27,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A27,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F27" s="10">
@@ -2245,11 +2277,11 @@
         <v>113.3</v>
       </c>
       <c r="D28" s="10">
-        <f>FORECAST.LINEAR(A28,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A28,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E28" s="10">
-        <f>FORECAST.ETS(A28,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A28,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F28" s="10">
@@ -2275,11 +2307,11 @@
         <v>72.7</v>
       </c>
       <c r="D29" s="10">
-        <f>FORECAST.LINEAR(A29,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A29,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E29" s="10">
-        <f>FORECAST.ETS(A29,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A29,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F29" s="10">
@@ -2305,11 +2337,11 @@
         <v>67.8</v>
       </c>
       <c r="D30" s="10">
-        <f>FORECAST.LINEAR(A30,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A30,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E30" s="10">
-        <f>FORECAST.ETS(A30,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A30,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F30" s="10">
@@ -2335,11 +2367,11 @@
         <v>75.8</v>
       </c>
       <c r="D31" s="10">
-        <f>FORECAST.LINEAR(A31,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A31,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E31" s="10">
-        <f>FORECAST.ETS(A31,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A31,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F31" s="10">
@@ -2365,11 +2397,11 @@
         <v>81.59999999999999</v>
       </c>
       <c r="D32" s="10">
-        <f>FORECAST.LINEAR(A32,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A32,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E32" s="10">
-        <f>FORECAST.ETS(A32,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A32,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F32" s="10">
@@ -2395,11 +2427,11 @@
         <v>89.8</v>
       </c>
       <c r="D33" s="10">
-        <f>FORECAST.LINEAR(A33,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A33,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E33" s="10">
-        <f>FORECAST.ETS(A33,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A33,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F33" s="10">
@@ -2425,11 +2457,11 @@
         <v>92.40000000000001</v>
       </c>
       <c r="D34" s="10">
-        <f>FORECAST.LINEAR(A34,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A34,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E34" s="10">
-        <f>FORECAST.ETS(A34,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A34,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F34" s="10">
@@ -2455,11 +2487,11 @@
         <v>95.8</v>
       </c>
       <c r="D35" s="10">
-        <f>FORECAST.LINEAR(A35,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A35,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E35" s="10">
-        <f>FORECAST.ETS(A35,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A35,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F35" s="10">
@@ -2485,11 +2517,11 @@
         <v>94.3</v>
       </c>
       <c r="D36" s="10">
-        <f>FORECAST.LINEAR(A36,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A36,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E36" s="10">
-        <f>FORECAST.ETS(A36,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A36,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F36" s="10">
@@ -2515,11 +2547,11 @@
         <v>88.2</v>
       </c>
       <c r="D37" s="10">
-        <f>FORECAST.LINEAR(A37,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A37,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E37" s="10">
-        <f>FORECAST.ETS(A37,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A37,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F37" s="10">
@@ -2545,11 +2577,11 @@
         <v>88.5</v>
       </c>
       <c r="D38" s="10">
-        <f>FORECAST.LINEAR(A38,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A38,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E38" s="10">
-        <f>FORECAST.ETS(A38,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A38,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F38" s="10">
@@ -2575,11 +2607,11 @@
         <v>103</v>
       </c>
       <c r="D39" s="10">
-        <f>FORECAST.LINEAR(A39,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A39,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E39" s="10">
-        <f>FORECAST.ETS(A39,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A39,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F39" s="10">
@@ -2605,11 +2637,11 @@
         <v>127</v>
       </c>
       <c r="D40" s="10">
-        <f>FORECAST.LINEAR(A40,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A40,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E40" s="10">
-        <f>FORECAST.ETS(A40,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A40,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F40" s="10">
@@ -2637,11 +2669,11 @@
         </is>
       </c>
       <c r="D41" s="12">
-        <f>FORECAST.LINEAR(A41,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A41,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E41" s="12">
-        <f>FORECAST.ETS(A41,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A41,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F41" s="13" t="n"/>
@@ -2666,11 +2698,11 @@
         </is>
       </c>
       <c r="D42" s="12">
-        <f>FORECAST.LINEAR(A42,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A42,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E42" s="12">
-        <f>FORECAST.ETS(A42,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A42,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F42" s="13" t="n"/>
@@ -2695,11 +2727,11 @@
         </is>
       </c>
       <c r="D43" s="12">
-        <f>FORECAST.LINEAR(A43,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A43,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E43" s="12">
-        <f>FORECAST.ETS(A43,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A43,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F43" s="13" t="n"/>
@@ -2724,11 +2756,11 @@
         </is>
       </c>
       <c r="D44" s="12">
-        <f>FORECAST.LINEAR(A44,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A44,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E44" s="12">
-        <f>FORECAST.ETS(A44,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A44,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F44" s="13" t="n"/>
@@ -2753,11 +2785,11 @@
         </is>
       </c>
       <c r="D45" s="12">
-        <f>FORECAST.LINEAR(A45,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A45,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E45" s="12">
-        <f>FORECAST.ETS(A45,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A45,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F45" s="13" t="n"/>
@@ -2782,11 +2814,11 @@
         </is>
       </c>
       <c r="D46" s="12">
-        <f>FORECAST.LINEAR(A46,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A46,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E46" s="12">
-        <f>FORECAST.ETS(A46,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A46,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F46" s="13" t="n"/>
@@ -2811,11 +2843,11 @@
         </is>
       </c>
       <c r="D47" s="12">
-        <f>FORECAST.LINEAR(A47,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A47,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E47" s="12">
-        <f>FORECAST.ETS(A47,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A47,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F47" s="13" t="n"/>
@@ -2840,11 +2872,11 @@
         </is>
       </c>
       <c r="D48" s="12">
-        <f>FORECAST.LINEAR(A48,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A48,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E48" s="12">
-        <f>FORECAST.ETS(A48,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A48,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F48" s="13" t="n"/>
@@ -2869,11 +2901,11 @@
         </is>
       </c>
       <c r="D49" s="12">
-        <f>FORECAST.LINEAR(A49,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A49,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E49" s="12">
-        <f>FORECAST.ETS(A49,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A49,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F49" s="13" t="n"/>
@@ -2898,11 +2930,11 @@
         </is>
       </c>
       <c r="D50" s="12">
-        <f>FORECAST.LINEAR(A50,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A50,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E50" s="12">
-        <f>FORECAST.ETS(A50,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A50,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F50" s="13" t="n"/>
@@ -2927,11 +2959,11 @@
         </is>
       </c>
       <c r="D51" s="12">
-        <f>FORECAST.LINEAR(A51,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A51,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E51" s="12">
-        <f>FORECAST.ETS(A51,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A51,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F51" s="13" t="n"/>
@@ -2956,11 +2988,11 @@
         </is>
       </c>
       <c r="D52" s="12">
-        <f>FORECAST.LINEAR(A52,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
+        <f>FORECAST(A52,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40)</f>
         <v/>
       </c>
       <c r="E52" s="12">
-        <f>FORECAST.ETS(A52,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
+        <f>_xlfn.FORECAST.ETS(A52,Historical_Data!$C$5:$C$40,Historical_Data!$A$5:$A$40,12)</f>
         <v/>
       </c>
       <c r="F52" s="13" t="n"/>
@@ -2970,6 +3002,7 @@
         </is>
       </c>
     </row>
+    <row r="53"/>
     <row r="54" ht="24" customHeight="1">
       <c r="A54" s="15" t="inlineStr">
         <is>
@@ -2998,6 +3031,9 @@
           <t>Interpretation</t>
         </is>
       </c>
+      <c r="E55" s="25" t="n"/>
+      <c r="F55" s="25" t="n"/>
+      <c r="G55" s="26" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="17" t="inlineStr">
@@ -3019,6 +3055,9 @@
           <t>Average error of the straight-line trend fit.</t>
         </is>
       </c>
+      <c r="E56" s="25" t="n"/>
+      <c r="F56" s="25" t="n"/>
+      <c r="G56" s="26" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="20" t="inlineStr">
@@ -3040,6 +3079,9 @@
           <t>Average error of the trend+seasonality model. Usually lower.</t>
         </is>
       </c>
+      <c r="E57" s="25" t="n"/>
+      <c r="F57" s="25" t="n"/>
+      <c r="G57" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3077,6 +3119,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -3170,7 +3213,7 @@
         </is>
       </c>
       <c r="C6" s="22">
-        <f>FORECAST.LINEAR(future_x, known_ys, known_xs)
+        <f>FORECAST(future_x, known_ys, known_xs)
 Future_x = future period number</f>
         <v/>
       </c>
@@ -3197,7 +3240,7 @@
         </is>
       </c>
       <c r="C7" s="23">
-        <f>FORECAST.ETS(target_date, values, timeline, seasonality)
+        <f>_xlfn.FORECAST.ETS(target_date, values, timeline, seasonality)
 Seasonality: 12 for monthly, 4 for quarterly</f>
         <v/>
       </c>
@@ -3224,7 +3267,7 @@
         </is>
       </c>
       <c r="C8" s="22">
-        <f>FORECAST.ETS.CONFINT(target, values, timeline, confidence_level, seasonality)
+        <f>_xlfn.FORECAST.ETS.CONFINT(target, values, timeline, confidence_level, seasonality)
 0.95 = 95% confidence interval</f>
         <v/>
       </c>
@@ -3374,6 +3417,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="50" customHeight="1">
       <c r="A15" s="24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix corrupted sheet3: store formula-syntax examples as text strings (not real formulas)
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-12/06_Forecasting.xlsx
+++ b/rFLA300/chapter-12/06_Forecasting.xlsx
@@ -613,7 +613,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1536,7 +1535,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3002,7 +3000,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
     <row r="54" ht="24" customHeight="1">
       <c r="A54" s="15" t="inlineStr">
         <is>
@@ -3119,7 +3116,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -3212,10 +3208,11 @@
           <t>Extends historical data using linear regression (Y = mx + b).</t>
         </is>
       </c>
-      <c r="C6" s="22">
-        <f>FORECAST(future_x, known_ys, known_xs)
-Future_x = future period number</f>
-        <v/>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> =FORECAST(x, known_ys, known_xs)
+x = future period number</t>
+        </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
@@ -3239,10 +3236,11 @@
           <t>Exponential Triple Smoothing — models level + trend + seasonality.</t>
         </is>
       </c>
-      <c r="C7" s="23">
-        <f>_xlfn.FORECAST.ETS(target_date, values, timeline, seasonality)
-Seasonality: 12 for monthly, 4 for quarterly</f>
-        <v/>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> =FORECAST.ETS(target_date, values, timeline, seasonality)
+Seasonality: 12 for monthly, 4 for quarterly</t>
+        </is>
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
@@ -3266,10 +3264,11 @@
           <t>Generates a confidence interval around the ETS forecast.</t>
         </is>
       </c>
-      <c r="C8" s="22">
-        <f>_xlfn.FORECAST.ETS.CONFINT(target, values, timeline, confidence_level, seasonality)
-0.95 = 95% confidence interval</f>
-        <v/>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> =FORECAST.ETS.CONFINT(target, values, timeline, confidence, seasonality)
+confidence: 0.95 = 95% interval</t>
+        </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
@@ -3348,9 +3347,11 @@
           <t>Average of |actual - predicted| — lower is better.</t>
         </is>
       </c>
-      <c r="C11" s="23">
-        <f>AVERAGE(ABS(actuals - forecasts))</f>
-        <v/>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> =AVERAGE(ABS(actuals_range - forecasts_range))
+where actuals and forecasts are cell ranges</t>
+        </is>
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
@@ -3417,7 +3418,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="50" customHeight="1">
       <c r="A15" s="24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix sheet3 XML corruption: rewrite Forecasting_Concepts with no formula-starting values
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-12/06_Forecasting.xlsx
+++ b/rFLA300/chapter-12/06_Forecasting.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,8 +54,27 @@
       <name val="Courier New"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -107,8 +126,13 @@
         <fgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -150,11 +174,69 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -222,6 +304,27 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3102,326 +3205,321 @@
   <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Forecasting Concepts and Best Practices (Objective 9)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>Concept</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>What It Means</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Excel Implementation</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>Excel Function / Syntax</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
         <is>
           <t>When to Use</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="28" t="inlineStr">
         <is>
           <t>Business Example</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="17" t="inlineStr">
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Trend</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>The long-term upward or downward direction in the data.</t>
-        </is>
-      </c>
-      <c r="C4" s="22" t="inlineStr">
-        <is>
-          <t>FORECAST.LINEAR — fits a straight line through historical data</t>
-        </is>
-      </c>
-      <c r="D4" s="19" t="inlineStr">
-        <is>
-          <t>Data has clear upward/downward movement, no strong seasonality</t>
-        </is>
-      </c>
-      <c r="E4" s="19" t="inlineStr">
-        <is>
-          <t>Annual revenue growing steadily at 8% per year</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>Long-term upward or downward direction in data.</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>FORECAST(x, known_ys, known_xs)</t>
+        </is>
+      </c>
+      <c r="D4" s="30" t="inlineStr">
+        <is>
+          <t>Data has clear movement, no strong seasonality.</t>
+        </is>
+      </c>
+      <c r="E4" s="30" t="inlineStr">
+        <is>
+          <t>Annual revenue growing 8% per year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>Seasonality</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>Regular, repeating patterns within a fixed cycle (usually 12 months).</t>
-        </is>
-      </c>
-      <c r="C5" s="23" t="inlineStr">
-        <is>
-          <t>FORECAST.ETS with seasonality=12 — automatically detects and projects seasonal waves</t>
-        </is>
-      </c>
-      <c r="D5" s="21" t="inlineStr">
-        <is>
-          <t>Data repeats similar patterns every year (retail, tourism, agriculture)</t>
-        </is>
-      </c>
-      <c r="E5" s="21" t="inlineStr">
-        <is>
-          <t>High sales in Dec, low in Feb every year</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>FORECAST.LINEAR</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Extends historical data using linear regression (Y = mx + b).</t>
-        </is>
-      </c>
-      <c r="C6" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> =FORECAST(x, known_ys, known_xs)
-x = future period number</t>
-        </is>
-      </c>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>Simple trend with no strong seasonality</t>
-        </is>
-      </c>
-      <c r="E6" s="19" t="inlineStr">
-        <is>
-          <t>Projecting unit sales 6 months ahead when trend is stable</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="B5" s="32" t="inlineStr">
+        <is>
+          <t>Regular repeating patterns within a fixed cycle (usually 12 months).</t>
+        </is>
+      </c>
+      <c r="C5" s="32" t="inlineStr">
+        <is>
+          <t>FORECAST.ETS with seasonality=12</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
+        <is>
+          <t>Data repeats similar patterns every year.</t>
+        </is>
+      </c>
+      <c r="E5" s="32" t="inlineStr">
+        <is>
+          <t>High sales in Dec, low in Feb every year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>FORECAST (Linear)</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>Extends historical data using linear regression: Y = mx + b.</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>Syntax: FORECAST(x, known_ys, known_xs)  |  x = future period number</t>
+        </is>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>Simple trend with no strong seasonality.</t>
+        </is>
+      </c>
+      <c r="E6" s="30" t="inlineStr">
+        <is>
+          <t>Projecting unit sales 6 months ahead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>FORECAST.ETS</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>Exponential Triple Smoothing — models level + trend + seasonality.</t>
-        </is>
-      </c>
-      <c r="C7" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> =FORECAST.ETS(target_date, values, timeline, seasonality)
-Seasonality: 12 for monthly, 4 for quarterly</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>Data with BOTH trend AND seasonal variation</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>Monthly retail revenue with holiday spikes</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>Exponential Triple Smoothing: models level + trend + seasonality.</t>
+        </is>
+      </c>
+      <c r="C7" s="32" t="inlineStr">
+        <is>
+          <t>Syntax: FORECAST.ETS(target, values, timeline, seasonality)  |  seasonality: 12=monthly, 4=quarterly</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
+        <is>
+          <t>Data has BOTH trend AND seasonal variation.</t>
+        </is>
+      </c>
+      <c r="E7" s="32" t="inlineStr">
+        <is>
+          <t>Monthly retail revenue with holiday spikes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>FORECAST.ETS.CONFINT</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>Generates a confidence interval around the ETS forecast.</t>
         </is>
       </c>
-      <c r="C8" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> =FORECAST.ETS.CONFINT(target, values, timeline, confidence, seasonality)
-confidence: 0.95 = 95% interval</t>
-        </is>
-      </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>When you need to communicate forecast uncertainty</t>
-        </is>
-      </c>
-      <c r="E8" s="19" t="inlineStr">
-        <is>
-          <t>Report best case / worst case scenarios to leadership</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>Syntax: FORECAST.ETS.CONFINT(target, values, timeline, confidence, seasonality)  |  confidence=0.95 for 95%</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>When you need to communicate forecast uncertainty.</t>
+        </is>
+      </c>
+      <c r="E8" s="30" t="inlineStr">
+        <is>
+          <t>Best case / worst case scenarios for leadership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Moving Average</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>Smooths out noise by averaging the last N periods.</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>No built-in function — calculate with =AVERAGE(last N rows)
-ToolPak: Moving Average tool</t>
-        </is>
-      </c>
-      <c r="D9" s="21" t="inlineStr">
-        <is>
-          <t>Data is noisy; want to see underlying trend</t>
-        </is>
-      </c>
-      <c r="E9" s="21" t="inlineStr">
-        <is>
-          <t>Average last 3 months of sales to smooth week-to-week variation</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="C9" s="32" t="inlineStr">
+        <is>
+          <t>Syntax: AVERAGE(last N rows)  |  or use ToolPak: Data &gt; Data Analysis &gt; Moving Average</t>
+        </is>
+      </c>
+      <c r="D9" s="32" t="inlineStr">
+        <is>
+          <t>Data is noisy; want to see underlying trend.</t>
+        </is>
+      </c>
+      <c r="E9" s="32" t="inlineStr">
+        <is>
+          <t>Average last 3 months of sales to remove noise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>Holdout Validation</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>Using part of historical data to test forecast accuracy.</t>
-        </is>
-      </c>
-      <c r="C10" s="22" t="inlineStr">
-        <is>
-          <t>Reserve last 6–12 rows as a 'test set'; train on earlier rows; compare predictions to actuals</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>Always — before trusting any forecast model</t>
-        </is>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>Train on months 1-30, forecast months 31-36, measure error</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>Using part of historical data to test forecast accuracy before forecasting the future.</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>Reserve last 6-12 rows as a test set. Train on earlier rows. Compare predictions to actuals.</t>
+        </is>
+      </c>
+      <c r="D10" s="30" t="inlineStr">
+        <is>
+          <t>Always — before trusting any forecast model.</t>
+        </is>
+      </c>
+      <c r="E10" s="30" t="inlineStr">
+        <is>
+          <t>Train on months 1-30, test on 31-36, measure error.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Mean Absolute Error (MAE)</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
-        <is>
-          <t>Average of |actual - predicted| — lower is better.</t>
-        </is>
-      </c>
-      <c r="C11" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> =AVERAGE(ABS(actuals_range - forecasts_range))
-where actuals and forecasts are cell ranges</t>
-        </is>
-      </c>
-      <c r="D11" s="21" t="inlineStr">
-        <is>
-          <t>Evaluating and comparing forecast models</t>
-        </is>
-      </c>
-      <c r="E11" s="21" t="inlineStr">
-        <is>
-          <t>FORECAST.ETS MAE=$3.2K vs LINEAR MAE=$4.8K → ETS wins</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="B11" s="32" t="inlineStr">
+        <is>
+          <t>Average of |actual minus predicted|. Lower is better.</t>
+        </is>
+      </c>
+      <c r="C11" s="32" t="inlineStr">
+        <is>
+          <t>Syntax: AVERAGE(ABS(actuals_range - forecasts_range))  |  enter with Ctrl+Shift+Enter</t>
+        </is>
+      </c>
+      <c r="D11" s="32" t="inlineStr">
+        <is>
+          <t>Evaluating and comparing forecast models.</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="inlineStr">
+        <is>
+          <t>ETS MAE=3200 vs LINEAR MAE=4800. ETS wins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>Forecast Horizon</t>
         </is>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B12" s="30" t="inlineStr">
         <is>
           <t>How far into the future you are projecting.</t>
         </is>
       </c>
-      <c r="C12" s="22" t="inlineStr">
-        <is>
-          <t>Any future period number in FORECAST functions</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>Planning cycle length</t>
-        </is>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>Quarterly planning = 3-month horizon; annual budget = 12-month horizon</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>Any future period number passed to FORECAST or FORECAST.ETS.</t>
+        </is>
+      </c>
+      <c r="D12" s="30" t="inlineStr">
+        <is>
+          <t>Determined by your planning cycle length.</t>
+        </is>
+      </c>
+      <c r="E12" s="30" t="inlineStr">
+        <is>
+          <t>Quarterly planning = 3-month horizon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="52" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Extrapolation Risk</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
-        <is>
-          <t>Forecasts degrade in accuracy the further you project.</t>
-        </is>
-      </c>
-      <c r="C13" s="23" t="inlineStr">
-        <is>
-          <t>Compare 1-month vs 12-month ahead forecast errors</t>
-        </is>
-      </c>
-      <c r="D13" s="21" t="inlineStr">
-        <is>
-          <t>Always — be more cautious about longer forecasts</t>
-        </is>
-      </c>
-      <c r="E13" s="21" t="inlineStr">
-        <is>
-          <t>Do not blindly project 5 years using 2 years of data</t>
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>Forecasts degrade in accuracy the further out you project.</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="inlineStr">
+        <is>
+          <t>Compare 1-month vs 12-month ahead errors to see accuracy drop-off.</t>
+        </is>
+      </c>
+      <c r="D13" s="32" t="inlineStr">
+        <is>
+          <t>Always be more cautious about longer-range forecasts.</t>
+        </is>
+      </c>
+      <c r="E13" s="32" t="inlineStr">
+        <is>
+          <t>Do not project 5 years from only 2 years of data.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="50" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
-        <is>
-          <t>✏️ Practice Challenge: Using the FORECAST_Functions sheet, which model (LINEAR or ETS) has a lower MAE? Why do you think one outperforms the other on this dataset? Change the season argument in FORECAST.ETS from 12 to 1 — what happens to the forecast?</t>
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>Practice Challenge: Using the FORECAST_Functions sheet, which model (LINEAR or ETS) has a lower MAE? Why does one outperform the other? Change the seasonality argument in FORECAST.ETS from 12 to 1 and observe how the forecast values change.</t>
         </is>
       </c>
     </row>

</xml_diff>